<commit_message>
Add category field to publication and update execution counts in markdown_generator
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10469826_polimi_it/Documents/Dottorato/Curriculum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_F25DC773A252ABDACC10486189DB5B345BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{287770FC-9DC3-4394-ADDD-CF46A2DE2F23}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_F25DC773A252ABDACC10486189DB5B345BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D015DAAA-3DD4-4A9D-87C6-A867BFF61B29}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>pub_date</t>
   </si>
@@ -67,6 +67,12 @@
   </si>
   <si>
     <t>Bertoldo, N., Qureshi, T., Simpkins, D., Arrigoni, A., &amp; Dotelli, G. (2024). Concrete with Organic Waste Materials as Aggregate Replacement. Applied Sciences, 14(1), 108. https://doi.org/10.3390/app14010108.</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>manuscripts</t>
   </si>
 </sst>
 </file>
@@ -399,15 +405,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="59.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -415,22 +422,25 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -438,24 +448,27 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{23E8F861-DA45-4554-979A-A60E32043170}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{23E8F861-DA45-4554-979A-A60E32043170}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>